<commit_message>
Auto update LeetCode leaderboard
</commit_message>
<xml_diff>
--- a/Students.xlsx
+++ b/Students.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$D$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sabareesh</t>
+          <t>sabareesh</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -477,11 +477,33 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>https://leetcode.com/u/sabareesh_karikalan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>922525106265</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sabarivasan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SabarivasanP</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/u/SabarivasanP/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D2"/>
+  <autoFilter ref="A1:D3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>